<commit_message>
Update processed tsv and xls with upgraded metapredict (v2 -> v3)
</commit_message>
<xml_diff>
--- a/data_analysis/data/mt_nucleoid_PTMs_list_P-sites_processed.xlsx
+++ b/data_analysis/data/mt_nucleoid_PTMs_list_P-sites_processed.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.946</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.609,0.681</t>
+          <t>0.789,0.543</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.365,0.176,0.716</t>
+          <t>0.323,0.321,0.65</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.91,0.919,0.91</t>
+          <t>0.923,0.928,0.877</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.753,0.679,0.036,0.06</t>
+          <t>0.919,0.673,0.058,0.049</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>0.893,0.899,0.846,0.885,0.086</t>
+          <t>0.839,0.8,0.691,0.813,0.175</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -906,12 +906,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>0.355,0.256,0.28,0.126,0.114</t>
+          <t>0.571,0.356,0.341,0.078,0.074</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Ordered,Ordered,Ordered,Ordered,Ordered</t>
+          <t>Disordered,Ordered,Ordered,Ordered,Ordered</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -978,12 +978,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>0.541,0.349,0.014,0.013,0.01,0.017</t>
+          <t>0.071,0.05,0.013,0.013,0.026,0.014</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Disordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
+          <t>Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>0.294,0.086,0.037,0.24,0.44,0.46</t>
+          <t>0.071,0.052,0.043,0.22,0.161,0.126</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>0.073,0.057,0.231,0.312,0.022,0.62,0.988</t>
+          <t>0.153,0.148,0.367,0.383,0.198,0.847,0.98</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>0.912,0.033,0.013,0.009,0.323,0.421,0.245</t>
+          <t>0.887,0.035,0.029,0.02,0.184,0.177,0.138</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>0.132,0.14,0.041,0.025,0.083,0.077,0.01,0.011</t>
+          <t>0.227,0.172,0.139,0.076,0.185,0.135,0.078,0.065</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1338,12 +1338,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>0.85,0.838,0.817,0.412,0.219,0.041,0.044,0.121</t>
+          <t>0.964,0.958,0.871,0.703,0.623,0.054,0.068,0.061</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Disordered,Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
+          <t>Disordered,Disordered,Disordered,Disordered,Disordered,Ordered,Ordered,Ordered</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>0.056,0.023,0.041,0.029,0.01,0.004,0.139,0.064,0.105,0.064</t>
+          <t>0.044,0.022,0.049,0.032,0.026,0.035,0.077,0.08,0.08,0.044</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>0.811,0.007,0.002,0.0,0.126,0.054,0.081,0.038,0.016,0,0.144</t>
+          <t>0.869,0.014,0.022,0.025,0.035,0.019,0.03,0.022,0.009,0.014,0.057</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>0.936,0.982,0.966,0.025,0.182,0.526,0.861,0.973,0.976,0.994,0.306</t>
+          <t>0.96,0.982,0.94,0.11,0.312,0.573,0.709,0.816,0.848,0.985,0.312</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>0.993,0.993,0.985,0.139,0.131,0.112,0.015,0.003,0.077,0.013,0.207,0.677</t>
+          <t>0.944,0.905,0.865,0.076,0.072,0.068,0.04,0.041,0.083,0.061,0.322,0.612</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>0.857,0.084,0.078,0.017,0.038,0.066,0.037,0.043,0.052,0.042,0.001,0.047</t>
+          <t>0.843,0.044,0.046,0.02,0.019,0.041,0.039,0.02,0.021,0.014,0.026,0.037</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>0.62,0.39,0.432,0.421,0.449,0.449,0.174,0.263,0.144,0.084,0.891,0.863</t>
+          <t>0.71,0.496,0.3,0.247,0.216,0.21,0.178,0.16,0.204,0.249,0.839,0.852</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>0.634,0.81,1,1,0.974,0.94,0.115,0.036,0.018,0.081,0.182,0.045,0.458</t>
+          <t>0.552,0.773,0.99,0.948,0.936,0.889,0.15,0.124,0.107,0.066,0.153,0.044,0.335</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1914,12 +1914,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>0.54,0.098,0.124,0.131,0.12,0.028,0.021,0.014,0.003,0.05,0.659,0.642,0.591</t>
+          <t>0.618,0.061,0.058,0.064,0.067,0.021,0.026,0.02,0.019,0.026,0.204,0.195,0.19</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Disordered,Disordered,Disordered</t>
+          <t>Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.933,0.944,0.935,0.935,0.92,0.901,0.914,0.907,0.882,0.874,0.858,0.739,0.491,0.043</t>
+          <t>0.973,0.976,0.959,0.967,0.975,0.935,0.904,0.846,0.78,0.729,0.701,0.6,0.484,0.03</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>1,0.254,0.022,0.118,0.052,0.078,0.087,0.083,0.095,0.085,0.691,0.697,0.791,0.764</t>
+          <t>0.956,0.416,0.055,0.115,0.053,0.093,0.089,0.075,0.106,0.052,0.751,0.794,0.761,0.735</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>0.528,0.172,0.07,0.052,0.018,0.034,0.009,0.133,0.044,0.025,0.092,0.058,0.225,0.196,0.154</t>
+          <t>0.803,0.35,0.052,0.051,0.025,0.041,0.034,0.138,0.04,0.044,0.085,0.122,0.11,0.111,0.11</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2202,12 +2202,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>0.334,0.19,0.075,0.024,0.019,0.011,0.055,0.039,0.062,0.076,0.113,0.331,0.419,0.412,0.287,0.075</t>
+          <t>0.515,0.303,0.053,0.027,0.027,0.03,0.044,0.036,0.019,0.021,0.021,0.078,0.089,0.092,0.09,0.037</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
+          <t>Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>0.906,0.844,0.437,0.337,0.333,0.267,0.368,0.283,0.381,0.401,0.411,0.358,0.441,0.394,0.361,0.115,0.021</t>
+          <t>0.807,0.72,0.075,0.08,0.081,0.081,0.093,0.097,0.127,0.127,0.123,0.151,0.076,0.073,0.118,0.08,0.023</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>0.979,0.962,0.909,0.663,0.566,0.305,0.089,0.06,0.014,0.102,0.116,0.016,0.012,0.028,0.013,0.026,0.017,0</t>
+          <t>0.932,0.916,0.807,0.611,0.565,0.433,0.066,0.059,0.062,0.132,0.111,0.042,0.033,0.033,0.038,0.038,0.051,0.019</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>0.283,0.22,0.286,0.273,0.026,0.077,0.076,0.232,0.088,0.09,0.071,0.147,0.047,0.087,0.014,0.005,0.103,0.28,0.268,0.22</t>
+          <t>0.376,0.203,0.238,0.074,0.064,0.098,0.121,0.143,0.055,0.054,0.053,0.129,0.038,0.071,0.086,0.083,0.091,0.322,0.398,0.419</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2490,12 +2490,12 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>0.884,0.732,0,0,0.008,0.087,0.08,0.082,0.073,0.097,0.193,0.186,0.184,0.113,0.088,0.074,0.116,0.025,0.187,0.194</t>
+          <t>0.917,0.428,0.0,0.0,0.0,0.038,0.061,0.062,0.066,0.062,0.066,0.07,0.066,0.078,0.083,0.082,0.049,0.08,0.103,0.113</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
+          <t>Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>0.827,0.773,0.822,0.835,0.833,0.84,0.859,0.917,0.909,0.819,0.973,0.969,0.97,0.972,0.958,0.981,0.912,0.851,0.381,0.033,0.015</t>
+          <t>0.918,0.917,0.93,0.928,0.952,0.968,0.957,0.976,0.976,0.949,0.985,0.981,0.987,0.981,0.948,0.936,0.777,0.718,0.403,0.034,0.034</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2634,12 +2634,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>0.994,0.907,0.874,0.558,0.326,0.263,0.247,0.014,0.176,0.022,0.239,0.157,0.015,0,0,0.121,0.039,0.114,0.027,0.013,0.027</t>
+          <t>0.916,0.805,0.79,0.627,0.558,0.526,0.233,0.048,0.101,0.042,0.1,0.099,0.023,0.024,0.064,0.101,0.033,0.065,0.065,0.08,0.123</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Disordered,Disordered,Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
+          <t>Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2706,12 +2706,12 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>0.962,0.871,0.541,0.223,0.216,0.358,0.309,0.858,0.897,0.912,0.927,0.931,0.929,0.953,0.959,0.95,0.673,0.646,0.794,0.594,0.822,0.869,0.214,0.137,0.059,0.053,0.004,0.051,0.023</t>
+          <t>0.911,0.85,0.657,0.517,0.453,0.41,0.557,0.849,0.875,0.898,0.922,0.932,0.944,0.963,0.948,0.839,0.48,0.363,0.364,0.526,0.641,0.665,0.144,0.092,0.076,0.071,0.066,0.077,0.058</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Disordered,Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
+          <t>Disordered,Disordered,Disordered,Disordered,Ordered,Ordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Ordered,Ordered,Ordered,Disordered,Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>1,0.972,0.835,0.092,0.092,0.102,0.033,0.033,0.025,0.025,0.031,0.016,0.059,0.056,0.043,0.016,0.009,0,0.058,0.072,0.064,0.054,0.046,0.046,0.085,0.065,0.057,0.034,0.026</t>
+          <t>0.904,0.899,0.758,0.078,0.073,0.035,0.026,0.024,0.024,0.021,0.024,0.01,0.016,0.015,0.014,0.018,0.021,0.024,0.033,0.032,0.031,0.03,0.05,0.058,0.09,0.081,0.079,0.092,0.043</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2850,12 +2850,12 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>0.469,0.443,0.059,0.001,0.003,0,0.037,0.053,0.045,0.052,0.053,0.029,0.059,0.017,0.012,0.018,0.085,0.079,0.091,0.088,0.082,0.073,0.051,0.032,0.093,0.074,0.08,0.124,0.203,0.179,0.163,0.066,0.049,0.069,0.099</t>
+          <t>0.809,0.768,0.22,0.017,0.009,0.002,0.022,0.019,0.02,0.017,0.018,0.018,0.019,0.009,0.009,0.009,0.02,0.036,0.033,0.034,0.038,0.036,0.035,0.021,0.02,0.053,0.056,0.052,0.132,0.135,0.11,0.029,0.027,0.037,0.18</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
+          <t>Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>1,1,0.574,0.556,0.283,0.009,0.177,0.239,0.044,0.048,0.049,0.039,0.092,0.018,0.021,0.035,0.089,0.076,0.029,0.023,0.085,0.169,0.077,0.106,0.107,0.112,0.093,0.079,0.069,0.184,0.071,0.041,0.049,0.046,0.087</t>
+          <t>0.945,0.921,0.779,0.709,0.122,0.045,0.134,0.14,0.076,0.067,0.048,0.056,0.05,0.052,0.061,0.063,0.058,0.061,0.039,0.036,0.098,0.091,0.145,0.135,0.136,0.138,0.138,0.139,0.112,0.133,0.104,0.047,0.06,0.082,0.072</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>0.794,0.287,0.08,0.021,0,0,0.023,0.028,0.018,0.007,0.006,0.056,0.004,0.012,0.008,0.017,0.089,0.036,0.021,0.039,0.035,0.033,0.04,0.037,0.107,0.086,0.034,0.0,0.035,0.034,0.032,0.007,0.098,0.228,0.257,0.38,0.334,0.27,0.03</t>
+          <t>0.892,0.37,0.113,0.071,0.017,0.017,0.037,0.042,0.026,0.021,0.027,0.035,0.038,0.04,0.042,0.044,0.054,0.054,0.06,0.042,0.039,0.039,0.028,0.03,0.063,0.073,0.072,0.021,0.023,0.025,0.026,0.025,0.125,0.132,0.14,0.158,0.186,0.156,0.073</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3066,12 +3066,12 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>0.955,0.963,0.936,0.934,0.908,0.752,0.329,0.218,0.158,0.146,0.103,0.06,0.015,0.061,0.035,0.034,0.035,0.003,0.091,0.012,0.059,0.089,0.037,0.012,0.022,0.082,0.078,0.073,0.032,0.026,0.134,0.103,0.092,0.094,0.069,0.031,0.644,0.735,0.375,0.159,0.356,0.338,0.346,0.9,0.996</t>
+          <t>0.896,0.886,0.912,0.9,0.888,0.839,0.586,0.085,0.08,0.081,0.084,0.07,0.058,0.046,0.041,0.042,0.041,0.048,0.066,0.023,0.043,0.077,0.061,0.052,0.051,0.069,0.071,0.072,0.048,0.077,0.076,0.1,0.106,0.071,0.07,0.079,0.519,0.639,0.339,0.252,0.469,0.516,0.532,0.796,0.942</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Disordered,Disordered</t>
+          <t>Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Disordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Ordered,Disordered,Disordered,Ordered,Ordered,Ordered,Disordered,Disordered,Disordered,Disordered</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">

</xml_diff>